<commit_message>
Modulacion y reordenamiento de archivos y correccion de errores menores
</commit_message>
<xml_diff>
--- a/BaseDeDatos/BaseDeDatos.xlsx
+++ b/BaseDeDatos/BaseDeDatos.xlsx
@@ -4,8 +4,8 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Productos" sheetId="2" r:id="rId2"/>
-    <sheet name="Trabajos" sheetId="3" r:id="rId3"/>
+    <sheet name="Trabajos" sheetId="2" r:id="rId2"/>
+    <sheet name="Productos" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -410,79 +410,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Categoría</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Nombre</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Precio</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Descripción</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1773204708788</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Filtro de Aceite</v>
-      </c>
-      <c r="C2" t="str">
-        <v>WO410</v>
-      </c>
-      <c r="D2">
-        <v>10000</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>1773229926866</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Aceite de Motor</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Helix HX7 x4L</v>
-      </c>
-      <c r="D3">
-        <v>60000</v>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -541,4 +469,90 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Categoría</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Nombre</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Precio</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Descripción</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1773204708788</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Filtro de Aceite</v>
+      </c>
+      <c r="C2" t="str">
+        <v>WO410</v>
+      </c>
+      <c r="D2">
+        <v>10000</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>1773229926866</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Aceite de Motor</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Helix HX7 x4L</v>
+      </c>
+      <c r="D3">
+        <v>60000</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>1773753690642</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Filtro de Combustible</v>
+      </c>
+      <c r="C4" t="str">
+        <v>FCI1304</v>
+      </c>
+      <c r="D4">
+        <v>40000</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>